<commit_message>
Add SABSA matrix layers and supporting documentation
- Introduced the Component layer (5-component.md) detailing ICT products and technologies relevant to the project.
- Added the Operational layer (6-operacional.md) focusing on service management and operational risk management.
- Created a README.md file to outline the structure and purpose of the SABSA matrix files.
- Updated the presentation (Presentacion.pdf) and the SABSA matrix Excel file (SABSA-Matriz.xlsx) to reflect the new layers.
- Developed a detailed script (guion.md) for the project presentation, summarizing key points and transitions between layers.
- Enhanced the build_xlsx.py script to read from the new markdown files and populate the Excel matrix accordingly.
</commit_message>
<xml_diff>
--- a/apps/project/out/SABSA-Matriz.xlsx
+++ b/apps/project/out/SABSA-Matriz.xlsx
@@ -673,19 +673,19 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22.28" customWidth="1" style="10" min="1" max="1"/>
-    <col width="48" customWidth="1" style="10" min="2" max="7"/>
-    <col width="48" customWidth="1" style="11" min="3" max="3"/>
-    <col width="48" customWidth="1" style="11" min="4" max="4"/>
-    <col width="48" customWidth="1" style="11" min="5" max="5"/>
-    <col width="48" customWidth="1" style="11" min="6" max="6"/>
-    <col width="48" customWidth="1" style="11" min="7" max="7"/>
+    <col width="52" customWidth="1" style="10" min="2" max="7"/>
+    <col width="52" customWidth="1" style="11" min="3" max="3"/>
+    <col width="52" customWidth="1" style="11" min="4" max="4"/>
+    <col width="52" customWidth="1" style="11" min="5" max="5"/>
+    <col width="52" customWidth="1" style="11" min="6" max="6"/>
+    <col width="52" customWidth="1" style="11" min="7" max="7"/>
     <col width="30" customWidth="1" style="10" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="11">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>MATRIZ SABSA para la Gerencia de Pagos Inmediatos (Bre-B) de NovaPay S.A.</t>
+          <t>MATRIZ SABSA — Proyecto «Vinculación a Bre-B como participante» de NovaPay S.A. (Gerencia de Pagos Inmediatos)</t>
         </is>
       </c>
     </row>
@@ -769,66 +769,79 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="255" customHeight="1" s="11">
+    <row r="4" ht="333" customHeight="1" s="11">
       <c r="A4" s="17" t="n"/>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>- Disponibilidad: El servicio de envío y recepción Bre-B debe operar 24/7/365 con una disponibilidad mínima del 99,95 %.
-- Inmediatez: Cada transferencia debe quedar acreditada al beneficiario en menos de 20 segundos, tal como lo exige el esquema Bre-B.
-- Confianza: Los fondos y los datos personales de los clientes deben estar protegidos, puesto que una sola filtración o estafa masiva afecta la reputación de la marca.
-- Crecimiento: Se busca aumentar el volumen transaccional por llaves y QR sin que la tasa de fraude supere 5 puntos básicos del valor transado.</t>
+          <t>- Confianza del cliente: Los fondos y los datos de los clientes son el activo principal; una estafa masiva o una filtración golpea más a la marca que cualquier caída.
+- Lanzamiento de Bre-B: Ofrecer en la app transferencias por llaves y pagos QR interoperables con todo el sistema financiero.
+- Crecimiento: Captar a quienes hoy usan efectivo y aportar al objetivo de duplicar los clientes activos en 2027.
+- Servicio siempre disponible: Que el cliente pueda pagar a cualquier hora y que el dinero llegue en segundos.
+- Fraude controlado: Crecer sin superar el tope de fraude que fija la Junta (5 puntos básicos del valor transado).
+- Cumplimiento: Operar dentro de las reglas del Banco de la República y de la SFC, porque sin cumplimiento no hay permiso para operar.
+- Reputación: Ser reconocidos por la seguridad de los pagos, como lo plantea la visión 2030.</t>
         </is>
       </c>
       <c r="C4" s="18" t="inlineStr">
         <is>
-          <t>- Oportunidad: Bre-B es interoperable y sin costo para el usuario, lo cual permite captar clientes de efectivo y competir con los bancos grandes.
-- Amenaza de fraude: Estafas por ingeniería social (fraude APP), toma de cuentas (ATO) por SIM swap, phishing y smishing, así como el uso de cuentas mula.
-- Amenaza a la disponibilidad: Ataques DDoS sobre el canal 24/7 y caídas del proveedor cloud o de la conexión con el Banco de la República.
-- Amenaza interna y de terceros: Empleados con privilegios excesivos, proveedores de software comprometidos (supply chain) y ransomware.
-- Cumplimiento: SFC (CE 007/2018 de ciberseguridad, hoy integrada en la Circular Básica Jurídica - CE 006/2025), Banco de la República (CRE DSP-465 de 2025, reglamentos del DICE y del MOL) y Ley 1581/2012 de protección de datos.</t>
+          <t>- Oportunidad, crecimiento: Bre-B ya suma más de 110 millones de llaves y 245 participantes; conectarse permite captar a quienes hoy usan efectivo.
+- Oportunidad, comercios: Los pagos QR abren una línea de negocio con comercios pequeños que hoy solo reciben efectivo.
+- Oportunidad, marca: Ser reconocidos como la opción segura en un mercado donde las estafas con Bre-B son noticia.
+- Oportunidad, eficiencia: Menos manejo de efectivo y transferencias entre entidades sin costo para el cliente.
+- Amenaza, fraude: Estafas por engaño, robo de cuentas y cuentas mula; el pago es inmediato e irrevocable.
+- Amenaza, caídas: Una caída se nota de inmediato; los principales participantes estuvieron entre 95,8 % y 99,0 % de disponibilidad en el primer semestre de 2026.
+- Amenaza, regulación: Incumplir las reglas del Banco de la República o de la SFC trae sanciones y puede frenar la operación.
+- Amenaza, datos y terceros: Filtración de datos personales (Ley 1581) y fallas o compromisos de los proveedores.</t>
         </is>
       </c>
       <c r="D4" s="18" t="inlineStr">
         <is>
-          <t>- Vinculación (onboarding): Apertura digital de cuenta con validación de identidad (KYC) y biometría.
-- Gestión de llaves: Inscripción, portabilidad y cancelación de llaves (celular, cédula, correo, alfanumérica) ante el DICE.
-- Envío y recepción: Resolución de la llave, autorización del cliente, envío al sistema de pagos y acreditación.
-- Pagos a comercios: Generación y lectura de códigos QR interoperables.
-- Conciliación y liquidación: Cuadre diario con el MOL del Banco de la República.
-- Gestión de disputas y fraude: Atención de reclamos, bloqueo de cuentas y devoluciones.</t>
+          <t>- Vinculación a Bre-B: Acuerdo con un sistema de pago (SPBVI) y habilitación de la cuenta de liquidación en el Banco de la República.
+- Desarrollo del producto: Construir llaves, transferencias y QR en la app, con la seguridad incluida desde el diseño.
+- Pruebas y certificación: Pruebas internas, de seguridad y de certificación con el sistema de pago antes de salir.
+- Aceptación: Marcha blanca con empleados y un grupo cerrado de clientes, y aprobación formal de los sponsors.
+- Operación de llaves y pagos: Inscribir, trasladar y bloquear llaves, y atender el envío y la recepción 24/7.
+- Prevención y atención del fraude: Detectar, bloquear y devolver según las reglas de Bre-B.
+- Conciliación, contabilidad y liquidez: Cuadre diario de lo que se mueve por Bre-B y fondos suficientes en la cuenta de liquidación.
+- Comercial, servicio al cliente y cumplimiento: Lanzamiento y vinculación de comercios, atención de reclamos y reportes a la SFC, al Banco de la República y a la UIAF.</t>
         </is>
       </c>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>- Junta Directiva y Presidencia (CEO).
-- Vicepresidencia de Pagos (Gerencia de Pagos Inmediatos Bre-B).
-- Vicepresidencia de Tecnología (Plataforma, Desarrollo, SRE).
-- Oficina del CISO (Seguridad de la Información y Ciberseguridad) y Gerencia de Prevención de Fraude.
-- Riesgos (SARO), Cumplimiento (SARLAFT) y Oficial de Protección de Datos.
-- Empresa extendida: Banco de la República (DICE, MOL), proveedor cloud, proveedor de biometría y operadores móviles.</t>
+          <t>- Sponsors: Junta Directiva, Presidencia y VP Comercial y de Pagos, que patrocinan el proyecto porque mueve el objetivo de crecimiento.
+- Dueño del proyecto: Gerencia de Pagos Inmediatos.
+- Seguridad transversal: La oficina del CISO reporta a Presidencia y no a Tecnología, para acompañar a todas las áreas sin conflicto de intereses.
+- Áreas de negocio: Comercial y Mercadeo, Operaciones, Contabilidad, Finanzas y Tesorería, y Servicio al cliente.
+- Áreas de soporte: Tecnología, Prevención de fraude, Jurídico y Talento humano (perfiles de cargo y formación).
+- Segunda línea de defensa: Riesgos (SIAR), Cumplimiento (SARLAFT) y Oficial de Protección de Datos.
+- Empresa extendida: Banco de la República (DICE y MOL), el sistema de pago al que se conecta, el proveedor de nube, la validación de identidad y los operadores móviles.
+- Clientes y entes de control: Personas y comercios; SFC y SIC.</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>- Sede principal: Oficinas en Bogotá (operación, SOC y atención al cliente).
-- Nube: Región cloud principal y región alterna (activo-pasivo), con datos de clientes colombianos bajo las reglas de transferencia internacional de la Ley 1581.
-- Conexión dedicada: Enlaces privados y redundantes hacia la infraestructura del Banco de la República.
-- Canales: App móvil (iOS y Android), web y API para comercios.
-- Jurisdicción: Colombia (vigilancia de la SFC y regulación del Banco de la República).</t>
+          <t>- Sede principal: Bogotá, donde están el equipo del proyecto, la operación y la atención al cliente.
+- Centros de datos: Uno principal y uno alterno del proveedor tecnológico, para no depender de un solo sitio.
+- Banco de la República: Donde se registran las llaves y se liquidan los pagos.
+- Canales: App móvil para personas y QR para comercios en todo el país.
+- Jurisdicción: Colombia, bajo la SFC, el Banco de la República y la SIC; si los datos se alojan fuera del país, aplican las reglas de transferencia internacional de datos.
+- Trabajo remoto: Parte del equipo trabaja desde casa, lo cual extiende el perímetro de la empresa.</t>
         </is>
       </c>
       <c r="G4" s="18" t="inlineStr">
         <is>
-          <t>- Operación continua: El servicio no tiene ventana de cierre, por lo cual todo mantenimiento debe hacerse sin interrupción.
-- Tiempo de transacción: Menos de 20 segundos de extremo a extremo.
-- Picos: Quincenas, primas y días festivos con hasta 5 veces el volumen promedio.
-- Reporte de incidentes: Los incidentes cibernéticos se reportan a la SFC y se informan a los clientes afectados en los plazos establecidos.
-- Liquidación: Ciclos de liquidación definidos por el MOL.</t>
+          <t>- Lanzamiento de Bre-B: La Junta lo necesita en el mercado en el cuarto trimestre de 2027, antes de la temporada decembrina.
+- Crecimiento: Duplicar los clientes activos a diciembre de 2027, con la captación medida mes a mes desde el lanzamiento.
+- Servicio siempre disponible: 24/7 desde el primer día, y cada pago en menos de 20 segundos (el Banco de la República lo exige en el 99,5 % de las operaciones).
+- Fraude controlado: Por debajo de 5 pb desde el lanzamiento, revisado cada mes por la Junta.
+- Confianza del cliente: Devolución por fraude en máximo 10 días de investigación y 2 días hábiles para devolver.
+- Cumplimiento: Reportes a la SFC y al Banco de la República en los plazos que fija cada norma.
+- Reputación: Ser reconocidos como la billetera más segura a 2030, como lo plantea la visión.</t>
         </is>
       </c>
       <c r="H4" s="19" t="inlineStr">
         <is>
-          <t>Junta Directiva - CEO - VP de Pagos - CISO</t>
+          <t>Junta Directiva - Presidencia - VP Comercial y de Pagos (sponsors)</t>
         </is>
       </c>
     </row>
@@ -879,67 +892,83 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="255" customHeight="1" s="11">
+    <row r="6" ht="294" customHeight="1" s="11">
       <c r="A6" s="17" t="n"/>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>- Disponible: Las transferencias deben poder hacerse a cualquier hora, porque el cliente espera que Bre-B funcione igual que el efectivo.
-- Confidencial: Los datos personales, los saldos y la relación llave-cuenta solo los conoce quien los necesita.
-- Íntegro: El monto, el destinatario y la cuenta no se pueden alterar entre la autorización del cliente y la liquidación.
-- Autenticado: Toda operación se ata a un cliente y a un dispositivo verificados.
-- No repudiable: Cada transferencia queda firmada y registrada, de forma que el cliente no pueda negar una operación legítima ni la empresa negar una reclamación válida.
-- Resistente al fraude y cumplido: Se detectan patrones anómalos en tiempo real y se demuestra el cumplimiento ante la SFC y el Banco de la República.</t>
+          <t>- Resistente al fraude (objetivo: fraude controlado): Se detecta el engaño antes de mover el dinero.
+- Disponible (objetivo: servicio siempre disponible): El servicio opera 24/7 y se recupera rápido ante una falla.
+- Autenticado (objetivo: confianza del cliente): Cada orden la da el titular verificado, desde un equipo de confianza.
+- Íntegro (objetivos: confianza y cumplimiento): El monto, el destinatario y la cuenta no se alteran entre la autorización y la liquidación.
+- Confidencial y privado (objetivos: confianza y reputación): Los datos personales, los saldos y la relación llave-cuenta solo los ve quien los necesita.
+- Oportuno (objetivo: servicio siempre disponible): El pago llega en menos de 20 segundos.
+- No repudiable (objetivo: cumplimiento): Queda evidencia de quién ordenó cada pago, lo que permite resolver devoluciones.
+- Cumplido (objetivo: cumplimiento): Se puede demostrar el cumplimiento ante el Banco de la República, la SFC y la SIC.</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>- Objetivo de control 1: Ninguna transferencia sin autenticación fuerte del cliente y sin un dispositivo vinculado.
-- Objetivo de control 2: Toda transacción pasa por un scoring de fraude antes de enviarse.
-- Objetivo de control 3: Los datos sensibles se cifran en tránsito y en reposo, con llaves bajo custodia de un HSM.
-- Objetivo de control 4: Recuperación del servicio dentro de los tiempos acordados ante cualquier incidente.
-- Arquitectura de políticas: Política general de seguridad (ISO 27001:2022), política de pagos inmediatos, política de gestión de llaves criptográficas, política de privacidad y política de desarrollo seguro.</t>
+          <t>- Objetivo 1: Ningún pago ni trámite de llaves sin autenticación fuerte del titular.
+- Objetivo 2: Todo pago se evalúa por riesgo de fraude antes de enviarse.
+- Objetivo 3: La información sensible se protege en todo su ciclo de vida (en tránsito, en reposo y en uso).
+- Objetivo 4: El servicio se recupera dentro de los tiempos que acepta el negocio, incluso ante un ciberataque.
+- Objetivo 5: El acceso a la información y a los sistemas es por mínimo privilegio y deja rastro.
+- Objetivo 6: Todo cambio al producto incluye seguridad desde el diseño.
+- Objetivo de habilitación: La seguridad no estorba la experiencia (menos de 20 s y pocos pasos), porque sin uso no hay crecimiento.
+- Arquitectura de políticas: Política general de seguridad, de pagos inmediatos, de privacidad, de desarrollo seguro, criptográfica, de terceros y de uso de IA.</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>- Zero Trust: No se confía por ubicación de red, sino que toda solicitud (cliente, servicio o empleado) se autentica y autoriza.
-- Defensa en profundidad: Controles en capas (dispositivo, red, aplicación, datos, monitoreo).
-- Privacy by design: Se minimiza el dato mostrado al resolver una llave (nombre parcialmente oculto) y se recolecta solo lo necesario.
-- DevSecOps: La seguridad se integra al ciclo de desarrollo (SDLC) con análisis automáticos en el pipeline.
-- Resiliencia: Arquitectura multi-zona y multi-región con conmutación automática.</t>
+          <t>- Zero Trust: Nadie es de confianza por estar «adentro»; se verifica cada solicitud de clientes, empleados y sistemas.
+- Defensa en profundidad: Varias capas de protección, de forma que si una falla la siguiente contiene el ataque.
+- Gestión del fraude como proceso continuo: Prevenir, detectar, bloquear, devolver y aprender.
+- Desarrollo seguro (DevSecOps): La seguridad entra en el ciclo de desarrollo desde el diseño y no al final.
+- Gestión de la información: Clasificar, proteger y eliminar la información según su valor.
+- Gestión de incidentes y comunicación: Responder, reportar a la SFC y avisar a los clientes afectados.
+- Resiliencia: El servicio se diseña para tolerar la caída de un sitio completo.
+- Privacidad desde el diseño e IA gobernada: Se recolecta solo lo necesario y se usa una sola IA corporativa autorizada.</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>- Dueño del proceso: VP de Pagos.
-- Dueño del riesgo de ciberseguridad: CISO.
-- Dueño del riesgo de fraude: Gerencia de Prevención de Fraude.
-- Custodios: Equipos de Plataforma (infraestructura y llaves) y de Datos.
-- Usuarios: Clientes personas y comercios, agentes de servicio al cliente y analistas de fraude.
-- Proveedores: Banco de la República, proveedor cloud, biometría, SMS/push y antifraude.</t>
+          <t>- Dueño del proceso: VP Comercial y de Pagos.
+- Dueños del riesgo: CISO (ciberseguridad) y Gerencia de Prevención de Fraude (fraude).
+- Administrador de la información: Cada dueño de proceso clasifica sus datos y decide quién accede a ellos.
+- Administradores técnicos (custodios): Administrador de la plataforma y la nube, administrador de accesos y administrador de bases de datos.
+- Áreas internas que prueban y aceptan: Operaciones, Servicio al cliente y Prevención de fraude validan antes de salir al público.
+- Usuarios internos: Agentes de servicio, analistas de fraude y desarrolladores.
+- Clientes: Personas y comercios.
+- Proveedores de servicio y contrapartes: Banco de la República, sistema de pago, nube y validación de identidad, bajo acuerdos de servicio y de seguridad.</t>
         </is>
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>- Dominio Cliente: App, dispositivo y canal de autenticación del cliente.
-- Dominio Exposición (DMZ): API Gateway, WAF y anti-DDoS.
-- Dominio Core de Pagos: Microservicios de llaves, envío, recepción y conciliación.
-- Dominio Datos sensibles: Bases de datos de clientes y transacciones, HSM/KMS.
-- Dominio Interbancario: Conexión con el DICE y el MOL.
-- Dominio Gestión: Accesos administrativos, SOC y herramientas corporativas.</t>
+          <t>- Banco de la República: Reglamento de pagos inmediatos (CRE DSP-465, versión del 31-mar-2026) y reglamentos del DICE y del MOL.
+- SFC, ciberseguridad: Circular Básica Jurídica (CE 006/2025), Parte I, Título IV, Capítulo V (antes CE 007/2018).
+- SFC, seguridad en canales: Requerimientos mínimos de seguridad y calidad, Parte I, Título II, Capítulo I.
+- Riesgo y lavado de activos: SIAR (riesgo operacional) y SARLAFT de la SFC.
+- Protección de datos: Ley 1581 de 2012 y hábeas data financiero (Ley 1266 de 2008).
+- ISO/IEC 27001:2022: Sistema de gestión de seguridad de la información (93 controles en 4 temas).
+- NIST CSF 2.0: Marco para gobernar, identificar, proteger, detectar, responder y recuperar.
+- OWASP, ISO 22301 e ISO/IEC 42001: Desarrollo seguro de la app y los servicios, continuidad del negocio y gestión de la IA.</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>- Marco de riesgo continuo: Se alinea con NIST CSF 2.0 (Gobernar, Identificar, Proteger, Detectar, Responder, Recuperar) y con el SARO de la SFC.
-- Revisión de riesgos: Trimestral, y de manera extraordinaria ante un incidente o un cambio en la regulación de Bre-B.
-- Indicadores (KRI): Tasa de fraude en pb, disponibilidad mensual, tiempo medio de detección (MTTD) y de respuesta (MTTR).
-- Ciclo de vida del dato: Desde la vinculación del cliente hasta la eliminación segura al terminar la retención legal.</t>
+          <t>- Marco de gestión de riesgos: ISO 31000 (proceso general de riesgos) e ISO/IEC 27005 (riesgos de seguridad de la información), alineados con el SIAR de la SFC.
+- Ciclo continuo: NIST CSF 2.0 (gobernar, identificar, proteger, detectar, responder y recuperar), con revisión trimestral e indicadores de riesgo.
+- Fraude por engaño: Seguimiento de anomalías en tiempo real y educación continua al cliente.
+- Robo de cuentas: Autenticación fuerte y bloqueo preventivo tras un cambio de equipo o de SIM.
+- Cuentas mula: Vigilancia de las cuentas que reciben y bloqueo de llaves por fraude.
+- Caída del servicio: Pruebas de continuidad y de recuperación cada semestre.
+- Vulnerabilidades e integridad: Hacking ético semestral (lo exige la SFC) y pruebas de validación de la información.
+- Accesos y terceros: Auditorías periódicas de accesos privilegiados y evaluación de proveedores.</t>
         </is>
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>CISO (Oficial de Seguridad de la Información)</t>
+          <t>CISO con los directores de área</t>
         </is>
       </c>
     </row>
@@ -990,68 +1019,80 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="307" customHeight="1" s="11">
+    <row r="8" ht="294" customHeight="1" s="11">
       <c r="A8" s="17" t="n"/>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>- Datos del cliente: Identificación, nombre, celular, correo, datos biométricos (plantilla, no imagen) y resultado de KYC.
-- Llaves Bre-B: Relación llave-cuenta registrada en el DICE.
-- Transacciones: ID, monto, origen, destino, hora, dispositivo, resultado del scoring.
-- Credenciales y secretos: Llaves criptográficas, certificados mTLS, tokens y secretos de aplicación.
-- Registros (logs): Eventos de autenticación, transacciones y accesos administrativos.</t>
+          <t>- Información transaccional: Pagos enviados y recibidos, montos, destinatarios y puntaje de fraude.
+- Información de clientes (clasificada): Identidad, biometría como plantilla, llaves y saldos.
+- Código fuente de la app y de los servicios: Si se altera o se filtra, se compromete todo el producto.
+- Motor de pagos y motor antifraude con su modelo de IA: Deciden si el dinero sale.
+- Servicio de llaves: Inscribe, traslada, bloquea y consulta llaves contra el DICE.
+- Conexión con el sistema de pago y el MOL: Canal por donde salen los pagos y se liquidan.
+- Llaves criptográficas, certificados y secretos: Su robo permitiría suplantar a NovaPay S.A. ante el sistema de pago.
+- Registros de auditoría y seguridad: Evidencia de cada operación y de cada acceso.</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>- Política de autenticación: Todo inicio de sesión y toda transferencia exigen MFA fuerte (passkey o biometría en el dispositivo vinculado), y el cambio de dispositivo o de celular bloquea las transferencias durante 24 horas.
-- Política de límites: Montos máximos por transacción y por día según el perfil de riesgo del cliente, ajustables solo con verificación adicional.
-- Política de llaves: Una llave no se inscribe ni se porta sin validar que el cliente es titular del celular o correo (código OTP) y sin notificación al canal anterior.
-- Política criptográfica: TLS 1.3 en todo canal externo, mTLS entre servicios y hacia el Banco de la República, cifrado AES-256 en reposo y llaves en HSM con rotación anual.
-- Política de acceso administrativo: Mínimo privilegio, acceso just-in-time aprobado por un segundo funcionario y sesiones grabadas.
-- Política de datos personales: Tratamiento conforme a la Ley 1581/2012 y la Ley 1266/2008 (habeas data financiero).</t>
+          <t>- Política de autenticación: Doble factor fuerte para entrar, para pagar y para todo trámite con llaves.
+- Política de límites transaccionales: Topes por perfil de riesgo, límite nocturno y tope bajo para equipos nuevos.
+- Política de gestión de llaves: Probar la titularidad antes de inscribir o trasladar, y avisar al canal anterior.
+- Política antifraude: Bloqueo de llaves por fraude y devolución según las reglas de Bre-B.
+- Política criptográfica: Todo canal cifrado y los datos sensibles cifrados en reposo, con llaves bajo custodia dedicada.
+- Política de acceso privilegiado: Mínimo privilegio, acceso temporal aprobado y sesiones grabadas.
+- Política de respaldo y recuperación: Copias protegidas contra borrado y pruebas periódicas de recuperación.
+- Políticas de soporte: Privacidad y retención de datos, desarrollo seguro, terceros y uso de IA.</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>- Flujo de un pago: Cliente se autentica, se resuelve la llave en el DICE, se muestra el nombre parcial del destinatario, se calcula el scoring de fraude, el cliente confirma y firma, se envía al sistema de pagos, se liquida en el MOL y se notifica a ambas partes.
-- Servicio de identidad (CIAM): Autenticación y gestión de dispositivos de los clientes.
-- Servicio de autorización: Políticas centralizadas para cada API.
-- Servicio de detección de fraude: Scoring en tiempo real con reglas y modelos.
-- Servicio criptográfico: Firma, cifrado y tokenización como servicio interno.
-- Servicio de monitoreo y auditoría: Correlación de eventos y trazabilidad de cada operación.</t>
+          <t>- Flujo de pago por llave: Autenticación fuerte → resolución de la llave con privacidad → antifraude → firma y no repudio → mensajería interbancaria segura → notificación.
+- Flujo de recepción de fondos: Antifraude de recepción (detección de cuentas mula) → notificación al cliente.
+- Flujo de inscripción o traslado de llave: Autenticación fuerte → verificación de titularidad → aviso al canal anterior.
+- Flujo de pago QR a comercio: Verificación de integridad del QR → antifraude → notificación.
+- Flujo de acceso administrativo: Gestión de accesos privilegiados → registro y monitoreo de la sesión.
+- Servicios transversales: Monitoreo y respuesta a incidentes, protección de datos, desarrollo seguro, continuidad, gestión de vulnerabilidades y seguridad de terceros.</t>
         </is>
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>- Modelo de confianza: El cliente confía en el dispositivo vinculado, la app confía solo en tokens emitidos por el CIAM y los servicios internos se confían entre sí solo con mTLS e identidad de servicio.
-- Perfil Cliente: Envía, recibe y administra sus propias llaves.
-- Perfil Agente de servicio: Consulta de datos enmascarados y bloqueo de cuentas, sin capacidad de mover dinero.
-- Perfil Analista de fraude: Revisión de alertas, retención y liberación de transacciones.
-- Perfil Ingeniero de plataforma: Acceso a infraestructura solo por just-in-time y sin acceso a datos de clientes en claro.
-- Perfil Auditor: Solo lectura de registros y evidencias.</t>
+          <t>- Cliente: Envía, recibe y administra solo sus propias llaves.
+- Comercio: Recibe pagos QR y consulta sus ventas.
+- Analista de fraude: Retiene, libera y marca transacciones; no administra sistemas.
+- Agente de servicio: Ve datos enmascarados y puede bloquear; no puede mover dinero.
+- Ingeniero de plataforma: Acceso temporal a la infraestructura, sin ver datos de clientes en claro.
+- Desarrollador: Solo ambientes de desarrollo y pruebas; nunca producción.
+- Auditor: Solo lectura de registros y evidencias.
+- Modelo de confianza: Nadie confía por defecto; cada usuario, equipo y servicio se identifica en cada solicitud.</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>- Cliente → Exposición: Solo HTTPS a través del API Gateway con WAF.
-- Exposición → Core: Solo llamadas autenticadas y autorizadas por política.
-- Core → Datos: Acceso por cuentas de servicio con permisos mínimos; ningún humano entra directo.
-- Core → Interbancario: Únicamente el servicio de mensajería Bre-B, por enlace dedicado con mTLS.
-- Gestión → todos: Solo vía bastión y acceso just-in-time.</t>
+          <t>- ISO 27001:2022, controles tecnológicos: Autenticación segura, criptografía, registro y monitoreo, desarrollo seguro, protección contra fuga de datos.
+- ISO 27001:2022, controles organizacionales: Políticas, relación con proveedores y servicios en la nube, gestión de incidentes, continuidad.
+- ISO 27001:2022, controles de personas y físicos: Concienciación, trabajo remoto y seguridad física delegada en el proveedor de nube.
+- CBJ, canales: Autenticación fuerte, perfil transaccional, pentest semestral, doble factor en móvil y gestión de riesgos del QR.
+- DSP-465: Nombre enmascarado, 20 segundos, bloqueo de llaves por fraude y devolución.
+- OWASP MASVS (app móvil): Almacenamiento, criptografía, autenticación, red, resiliencia y privacidad.
+- OWASP Top 10 de APIs: Autorización por objeto, autenticación, consumo de recursos y flujos de negocio sensibles.
+- Dominios de interacción: Cliente ↔ exposición ↔ core de pagos ↔ información sensible, y core ↔ interbancario; gestión entra solo por un punto controlado.</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
         <is>
-          <t>- Sesión del cliente: Expira tras 5 minutos de inactividad en la app.
-- Token de acceso: Vida de 10 minutos, con refresh atado al dispositivo.
-- Scoring de fraude: Debe responder en menos de 300 ms para no afectar la promesa de 20 segundos.
-- Retención: Registros transaccionales por 10 años (soporte contable) y logs de seguridad por al menos 2 años.
-- Rotación: Certificados mTLS cada 90 días y llaves de cifrado de datos cada año.</t>
+          <t>- Q1 2027: Autenticación fuerte, criptografía y gestión de accesos privilegiados listos, porque son la base de todo lo demás.
+- Q2 2027: Antifraude, gestión de llaves y mensajería interbancaria probados en la certificación con el sistema de pago.
+- Q2 2027: Pentest y análisis de vulnerabilidades antes de la marcha blanca.
+- Q3 2027: Monitoreo 24/7 (SOC) y playbooks de incidentes operando durante la marcha blanca.
+- Q4 2027: Prueba completa de recuperación antes del lanzamiento al público.
+- Vigencias de sesión: La sesión del cliente expira a los 5 minutos de inactividad y la credencial de acceso dura 10 minutos.
+- Tiempos de servicio: Resolución de llave ≤ 5 s, antifraude &lt; 300 ms y pago completo &lt; 20 s.</t>
         </is>
       </c>
       <c r="H8" s="19" t="inlineStr">
         <is>
-          <t>Arquitecto de Seguridad y Gerente de Pagos Inmediatos</t>
+          <t>CISO y Arquitecto de Seguridad</t>
         </is>
       </c>
     </row>
@@ -1100,65 +1141,80 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="216" customHeight="1" s="11">
+    <row r="10" ht="281" customHeight="1" s="11">
       <c r="A10" s="17" t="n"/>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>- Datos restringidos: Biometría, identificación, credenciales, llaves criptográficas (cifrado + tokenización).
-- Datos confidenciales: Saldos, transacciones, relación llave-cuenta (cifrado en reposo y enmascaramiento en consultas).
-- Datos internos: Métricas operativas y reportes agregados.
-- Datos públicos: Información comercial y tarifas.
-- Inventario: Catálogo de datos con dueño, clasificación, ubicación y tiempo de retención por cada tabla.</t>
+          <t>- Credenciales y biometría (restringido): Se guardan como plantillas cifradas, nunca como imágenes.
+- Llaves criptográficas (restringido): Solo viven dentro del HSM.
+- Identificación y número de cuenta (restringido): Se tokenizan fuera del dominio de datos sensibles.
+- Relación llave-cuenta (confidencial): Se cifra; al resolver una llave solo se muestra el nombre enmascarado.
+- Transacciones (confidencial): Monto, origen, destino, hora, dispositivo y puntaje de fraude.
+- Registros de auditoría (confidencial): Inmutables y con sello de tiempo confiable.
+- Código fuente (restringido): Repositorio privado, revisión obligatoria entre pares y commits firmados.
+- Catálogo de datos: Cada tabla con dueño, clasificación, ubicación y tiempo de retención.</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>- Reglas de fraude: Bloqueo automático si hay una nueva llave o un nuevo dispositivo con un monto alto, velocidad anómala o un destinatario reportado como mula.
-- Procedimiento de respuesta a incidentes: Playbooks para ATO, fuga de datos, DDoS y ransomware, con roles, escalamiento y reporte a la SFC.
-- Gestión de vulnerabilidades: Las vulnerabilidades críticas se corrigen en 7 días y las altas en 30.
-- Gestión de cambios: Todo cambio a producción pasa por revisión de código entre pares y por el pipeline seguro.
-- Continuidad: Plan de continuidad (BCP) y de recuperación (DRP) probados semestralmente.</t>
+          <t>- Reglas de fraude: Retener o bloquear si hay llave nueva, equipo nuevo con monto alto, velocidad anómala o destinatario marcado.
+- Reglas de límites: Límite nocturno, tope bajo durante 24 h para equipos nuevos y espera para subir los límites.
+- Bloqueo de llaves y devolución: Bloqueo inmediato ante fraude, investigación en ≤ 10 días y devolución en 2 días hábiles.
+- Playbooks de incidentes: Robo de cuentas, fraude masivo, DDoS, ransomware y caída del sistema de pago, con reporte a la SFC (taxonomía TUIC).
+- Gestión de vulnerabilidades: Las críticas se corrigen en 7 días y las altas en 30.
+- Gestión de cambios: Revisión entre pares, pipeline seguro y doble aprobación para producción.
+- Monitoreo de liquidez: Alerta temprana del saldo en el MOL para no quedar inactivo.
+- Fallo controlado del antifraude: Si el scoring no responde, el pago sigue con límites reducidos en vez de bloquearse todo.</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
         <is>
-          <t>- Device binding y passkeys (FIDO2): Llave privada en el enclave seguro del celular que firma cada transferencia.
-- API Gateway + WAF + anti-DDoS: Único punto de entrada desde internet.
-- mTLS y service mesh: Cifrado e identidad entre microservicios.
-- HSM/KMS: Generación y custodia de llaves, cifrado envolvente (envelope encryption) de las bases de datos.
-- Tokenización: Los números de cuenta y de identificación se sustituyen por tokens fuera del dominio de datos sensibles.
-- Motor de fraude en línea y SIEM: Decisión en tiempo real y correlación centralizada de eventos.</t>
+          <t>- Passkeys (FIDO2) y biometría con prueba de vida: Atadas al dispositivo vinculado (servicio de autenticación).
+- Motor antifraude en línea: Reglas + machine learning + biometría conductual (servicio antifraude).
+- HSM/KMS, cifrado envolvente y tokenización: Servicio de criptografía y protección de datos.
+- mTLS y firma de mensajes ISO 20022: Conexión con el sistema de pago (servicio de mensajería interbancaria).
+- WAF, anti-DDoS y gestión de bots: Servicio de protección perimetral.
+- Protección de la app: RASP, anti-tampering, detección de root/jailbreak y atestación del dispositivo.
+- SIEM con correlación y logs inmutables: Servicio de monitoreo, auditoría y no repudio.
+- DLP y EDR en los equipos de los empleados: Protección de endpoint y control de shadow AI.</t>
         </is>
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>- App del cliente: Login con biometría del celular (passkey), confirmación explícita con el nombre parcial del destinatario y alertas push de cada movimiento.
-- Consola interna: Inicio de sesión único (SSO) con MFA resistente a phishing (llave FIDO2) para todos los empleados.
-- Control de acceso: RBAC por perfil más reglas por atributo (ABAC) para montos y horarios.
-- Accesos privilegiados (PAM): Bóveda de credenciales y grabación de sesiones administrativas.</t>
+          <t>- App del cliente: Login biométrico, nombre enmascarado antes de confirmar y alerta push de cada movimiento.
+- Aviso antiestafa: La app aclara que en Bre-B no hay que «aceptar» transferencias para recibir dinero.
+- Consola interna: Inicio de sesión único con llave FIDO2 para todos los empleados.
+- Control de acceso: RBAC por perfil más reglas por atributo (ABAC) según monto, horario y ubicación.
+- Accesos privilegiados: Acceso temporal aprobado por un segundo funcionario, con la sesión grabada.
+- Protección de sesión: Bloqueo tras intentos fallidos, cierre por inactividad y aviso del último ingreso.</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>- Red: VPC por ambiente (desarrollo, pruebas, producción) totalmente separados.
-- Segmentación: Subredes por dominio (exposición, core, datos, interbancario, gestión) con listas de control entre ellas.
-- Plataforma: Contenedores en Kubernetes administrado, en tres zonas de disponibilidad.
-- Región alterna: Réplica de datos y de infraestructura como código lista para activar.
-- Enlaces al Banco de la República: Dos enlaces dedicados por proveedores distintos.</t>
+          <t>- Perímetro: WAF, anti-DDoS, CDN, lista blanca de IP y mTLS hacia el sistema de pago.
+- Red: Una VPC por ambiente y por dominio, subredes privadas sin salida directa a internet y microsegmentación.
+- Sistema operativo y contenedores: Imágenes mínimas firmadas, hardening CIS y seguridad en tiempo de ejecución.
+- Aplicación: Gateway con OAuth2, validación de esquemas, anti-replay e idempotencia.
+- Datos: Cifrado con llaves por dominio, tokenización y enmascaramiento fuera de producción.
+- Identidad: Passkeys para clientes, llave FIDO2 para empleados y gestión de accesos privilegiados.
+- Procedimental: Segregación de funciones, doble aprobación en producción y simulacros.
+- Sitios: Tres zonas de disponibilidad más una región alterna, y dos enlaces al sistema de pago.</t>
         </is>
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>- RTO del servicio de pagos: 15 minutos; RPO: 0 (sin pérdida de transacciones confirmadas).
-- Conmutación entre zonas: Automática, en menos de 1 minuto.
-- Sesión administrativa: Máximo 1 hora y cierre automático.
-- Backups: Continuos (punto en el tiempo) y copias inmutables diarias aisladas contra ransomware.
-- Bloqueo preventivo: 24 horas sin transferencias salientes tras cambio de dispositivo o SIM.</t>
+          <t>- Nivel 0 (pagos, antifraude, conexión): RTO menor a 1 minuto si cae una zona y de hasta 2 horas si cae la región; RPO 0.
+- Nivel 1 (llaves, notificaciones, QR): RTO de 1 hora; RPO de 5 minutos.
+- Nivel 2 (backoffice, analítica): RTO y RPO de 24 horas.
+- Ciberrecuperación: Copias inmutables aisladas, restaurando el último punto limpio en hasta 2 horas.
+- Latencias: Resolución de llave ≤ 5 s, antifraude &lt; 300 ms y pago completo &lt; 20 s.
+- Sesiones: El cliente se desconecta tras 5 minutos de inactividad y la sesión administrativa dura máximo 1 hora.
+- Bloqueo preventivo: 24 horas sin envíos tras un cambio de equipo o de SIM.</t>
         </is>
       </c>
       <c r="H10" s="19" t="inlineStr">
         <is>
-          <t>Director de Plataforma e Infraestructura Cloud</t>
+          <t>Director de Plataforma e Infraestructura</t>
         </is>
       </c>
     </row>
@@ -1205,59 +1261,67 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="164" customHeight="1" s="11">
+    <row r="12" ht="229" customHeight="1" s="11">
       <c r="A12" s="24" t="n"/>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>- Cómputo: Amazon EKS (Kubernetes) en la región principal y en la alterna.
-- Datos: Amazon Aurora PostgreSQL cifrado y Redis para caché de resolución de llaves.
-- Mensajería: Apache Kafka (Amazon MSK) para eventos de transacción.
-- Criptografía: AWS CloudHSM y AWS KMS.
-- Secretos: HashiCorp Vault.</t>
+          <t>- Repositorio transaccional: Amazon Aurora PostgreSQL cifrado (clientes, llaves y transacciones), con réplica entre regiones.
+- Repositorio de registros y evidencias: Amazon S3 con Object Lock en modo compliance (logs inmutables).
+- Repositorio de código: GitHub, con ramas protegidas y commits firmados (código de la app y de los servicios).
+- Caché de resolución de llaves: Redis (Amazon ElastiCache).
+- Procesamiento: Amazon EKS (Kubernetes) en la región principal y en la alterna.
+- Procesamiento de eventos: Apache Kafka (Amazon MSK).
+- Procesadores criptográficos y de secretos: AWS CloudHSM (raíz de confianza), AWS KMS y HashiCorp Vault.</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>- Detección de fraude: Feedzai (o equivalente) con reglas y modelos de machine learning.
+          <t>- Antifraude: Feedzai (o equivalente) con reglas y machine learning, gobernado bajo ISO/IEC 42001.
 - SIEM y SOAR: Microsoft Sentinel con playbooks automáticos.
-- Gestión de riesgos (GRC): Registro de riesgos y evidencias de cumplimiento en una herramienta GRC (p. ej. Archer).
-- Gestión de vulnerabilidades: Tenable para infraestructura y Snyk para dependencias y contenedores.
-- Postura cloud (CSPM): AWS Security Hub y GuardDuty.</t>
+- Postura en la nube: AWS Security Hub y Amazon GuardDuty.
+- Vulnerabilidades: Tenable para la infraestructura y Snyk para dependencias y contenedores.
+- Fuga de datos y shadow AI: Microsoft Purview DLP en los equipos y en la IA corporativa.
+- Registro de riesgos y cumplimiento: Herramienta GRC (p. ej. Archer) con el registro de riesgos y las evidencias.</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>- Protocolos: TLS 1.3, mTLS (certificados X.509), OAuth 2.1 / OpenID Connect, FIDO2/WebAuthn.
-- Mensajes Bre-B: Estándar ISO 20022 sobre el enlace dedicado.
-- Perímetro: Cloudflare (WAF, anti-DDoS y gestión de bots) delante del API Gateway.
-- Service mesh: Istio para mTLS automático.
-- Pipeline: GitHub Actions con Semgrep (SAST), Snyk (SCA), Trivy (contenedores) y OWASP ZAP (DAST).
+          <t>- Protocolos: TLS 1.3, mTLS (X.509), OAuth 2.1 / OpenID Connect y FIDO2/WebAuthn.
+- Mensajes con el sistema de pago: ISO 20022 sobre REST, como lo exige la DSP-465.
+- Perímetro: Cloudflare (WAF, anti-DDoS y bots) delante del API Gateway.
+- Service mesh: Istio, para mTLS automático entre microservicios.
+- Pipeline seguro: GitHub Actions con Semgrep (SAST), Snyk (SCA), Trivy (contenedores) y OWASP ZAP (DAST).
+- Protección de la app: SDK de RASP y atestación (Play Integrity / App Attest).
 - Endpoint: CrowdStrike Falcon en los equipos de los empleados.</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>- Identidad del cliente (CIAM): Auth0 / Okta Customer Identity o Keycloak.
+          <t>- Identidad de clientes (CIAM): Auth0 / Okta Customer Identity o Keycloak.
 - Identidad de empleados: Microsoft Entra ID con acceso condicional y llaves YubiKey.
-- PAM: CyberArk o Teleport para accesos just-in-time.
-- Roles: Analista de fraude, agente de servicio, ingeniero de plataforma, SRE, analista SOC, auditor, cada uno con su grupo y ACL en el directorio.</t>
+- Accesos privilegiados: CyberArk o Teleport para acceso temporal.
+- Roles y grupos: Analista de fraude, agente, ingeniero de plataforma, SRE, analista SOC y auditor, cada uno con su grupo y su ACL.
+- Ciclo de vida de identidades: Alta, cambio y baja automáticos desde el sistema de RR. HH.
+- Recertificación: Revisión trimestral de accesos por cada dueño de proceso.</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>- Nodos: Clústeres EKS de producción (3 zonas) y de DR en la región alterna.
-- Direccionamiento: Rangos de IP privados por VPC, sin IP pública en nodos de core ni de datos.
-- Puntos de intercambio: Endpoint de la API pública detrás de Cloudflare y conexión dedicada hacia el Banco de la República (AWS Direct Connect).
-- DNS: Registros internos en Route 53 privado y DNSSEC en el dominio público.</t>
+          <t>- Nodos: Clústeres EKS de producción en 3 zonas y clúster de DR en la región alterna.
+- Direccionamiento: Rangos de IP privados por VPC, sin IP pública en los nodos del core ni de datos.
+- Conexión al sistema de pago: AWS Direct Connect con dos enlaces por proveedores distintos.
+- Punto público: La API pública solo se expone detrás de Cloudflare.
+- DNS: Route 53 privado para lo interno y DNSSEC en el dominio público.</t>
         </is>
       </c>
       <c r="G12" s="18" t="inlineStr">
         <is>
-          <t>- Relojes: Sincronización NTP de todos los nodos (Amazon Time Sync) para que los logs y las firmas tengan sellos de tiempo confiables.
-- Pruebas de penetración: Trimestrales y antes de cada cambio mayor de la app.
-- Escaneo de vulnerabilidades: Semanal en infraestructura y en cada build en el pipeline.
-- Simulacros: Pruebas de DRP semestrales y ejercicios de mesa (tabletop) de ransomware anuales.
-- Rotación automática: Secretos de Vault diaria y certificados cada 90 días.</t>
+          <t>- Relojes: Sincronización NTP (Amazon Time Sync) en todos los nodos, para que logs y firmas tengan sellos de tiempo confiables.
+- Pentest: Semestral (exigencia de la SFC) y antes de cada cambio mayor de la app.
+- Escaneo de vulnerabilidades: Semanal en la infraestructura y en cada build del pipeline.
+- Simulacros: Pruebas de DRP semestrales y ejercicio de mesa de ransomware anual.
+- Rotación automática: Secretos de Vault a diario y certificados cada 90 días.
+- Recertificación de accesos: Trimestral.</t>
         </is>
       </c>
       <c r="H12" s="19" t="inlineStr">

</xml_diff>